<commit_message>
switch default answering prompt to v2 after side-by-side review
</commit_message>
<xml_diff>
--- a/eval/RBI_NBFC_Retrieval_Questions_results_v2.xlsx
+++ b/eval/RBI_NBFC_Retrieval_Questions_results_v2.xlsx
@@ -3435,12 +3435,12 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>answered a question the corpus should not cover - check for invention</t>
+          <t>correctly declined to answer</t>
         </is>
       </c>
       <c r="J55" t="n">

</xml_diff>